<commit_message>
Pulled newest version of manual variables
</commit_message>
<xml_diff>
--- a/data/labeling/rq4tlr-manual-variables.xlsx
+++ b/data/labeling/rq4tlr-manual-variables.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5027" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5025" uniqueCount="344">
   <si>
     <t>Done</t>
   </si>
@@ -830,13 +830,10 @@
     <t>The main subflow does not fulfill the use case implied by the name ("view emergency electronic health record")</t>
   </si>
   <si>
-    <t>Empty name. Steps 2 and 3 are not steps in the process, but constraints.</t>
+    <t>Steps 2 and 3 are not steps in the process, but constraints.</t>
   </si>
   <si>
-    <t>Empty name</t>
-  </si>
-  <si>
-    <t>Empty name. Steps 3-5 are not steps in the process, but constraints.</t>
+    <t>This flow should rather have the name "View appointments." Steps 3-5 are not steps in the process, but constraints.</t>
   </si>
   <si>
     <t>The first subflow of the use case does not describe a scenario that fulfills the implication of the use case name.</t>
@@ -881,10 +878,7 @@
     <t>Step 5 is a system-system interaction</t>
   </si>
   <si>
-    <t>No use case name. The final step contains a system-system interaction.</t>
-  </si>
-  <si>
-    <t>No use case name</t>
+    <t>The final step contains a system-system interaction.</t>
   </si>
   <si>
     <t>Step 4 only contains details. Steps 5-8 are parallel alternative paths.</t>
@@ -1483,8 +1477,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.13"/>
-    <col customWidth="1" min="2" max="2" width="7.25"/>
-    <col customWidth="1" min="3" max="3" width="9.88"/>
+    <col customWidth="1" min="2" max="2" width="7.88"/>
+    <col customWidth="1" min="3" max="3" width="10.13"/>
     <col customWidth="1" min="4" max="4" width="3.25"/>
     <col customWidth="1" min="5" max="5" width="7.0"/>
     <col customWidth="1" min="6" max="15" width="3.88"/>
@@ -5451,7 +5445,7 @@
         <v>0</v>
       </c>
       <c r="I82" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J82" s="5" t="b">
         <v>0</v>
@@ -5468,8 +5462,8 @@
       <c r="N82" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="O82" s="5" t="b">
-        <v>0</v>
+      <c r="O82" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>115</v>
@@ -7386,7 +7380,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H122" s="5" t="b">
         <v>0</v>
@@ -7436,7 +7430,7 @@
         <v>0</v>
       </c>
       <c r="G123" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H123" s="5" t="b">
         <v>0</v>
@@ -7532,7 +7526,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H125" s="5" t="b">
         <v>0</v>
@@ -7580,7 +7574,7 @@
         <v>0</v>
       </c>
       <c r="G126" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H126" s="5" t="b">
         <v>0</v>
@@ -10296,7 +10290,7 @@
         <v>0</v>
       </c>
       <c r="G182" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H182" s="5" t="b">
         <v>0</v>
@@ -10346,7 +10340,7 @@
         <v>0</v>
       </c>
       <c r="G183" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H183" s="5" t="b">
         <v>0</v>
@@ -10743,8 +10737,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.13"/>
-    <col customWidth="1" min="2" max="2" width="7.25"/>
-    <col customWidth="1" min="3" max="3" width="9.88"/>
+    <col customWidth="1" min="2" max="2" width="8.0"/>
+    <col customWidth="1" min="3" max="3" width="10.13"/>
     <col customWidth="1" min="4" max="4" width="3.25"/>
     <col customWidth="1" min="5" max="5" width="7.0"/>
     <col customWidth="1" min="6" max="15" width="3.88"/>
@@ -11286,8 +11280,8 @@
       <c r="N11" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="O11" s="5" t="b">
-        <v>0</v>
+      <c r="O11" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="P11" s="9" t="s">
         <v>244</v>
@@ -16665,7 +16659,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H122" s="5" t="b">
         <v>0</v>
@@ -16715,7 +16709,7 @@
         <v>0</v>
       </c>
       <c r="G123" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H123" s="5" t="b">
         <v>0</v>
@@ -16741,9 +16735,7 @@
       <c r="O123" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="P123" s="6" t="s">
-        <v>272</v>
-      </c>
+      <c r="P123" s="6"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="b">
@@ -16792,7 +16784,7 @@
         <v>1</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="125">
@@ -16815,7 +16807,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H125" s="5" t="b">
         <v>0</v>
@@ -16863,7 +16855,7 @@
         <v>0</v>
       </c>
       <c r="G126" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H126" s="5" t="b">
         <v>0</v>
@@ -16937,7 +16929,7 @@
         <v>0</v>
       </c>
       <c r="P127" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="128">
@@ -16987,7 +16979,7 @@
         <v>1</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="129">
@@ -17181,7 +17173,7 @@
         <v>1</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="133">
@@ -17375,7 +17367,7 @@
         <v>1</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="137">
@@ -17713,7 +17705,7 @@
         <v>1</v>
       </c>
       <c r="P143" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="144">
@@ -17763,7 +17755,7 @@
         <v>1</v>
       </c>
       <c r="P144" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="145">
@@ -18053,7 +18045,7 @@
         <v>1</v>
       </c>
       <c r="P150" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="151">
@@ -18103,7 +18095,7 @@
         <v>1</v>
       </c>
       <c r="P151" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="152">
@@ -18249,7 +18241,7 @@
         <v>1</v>
       </c>
       <c r="P154" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="155">
@@ -18347,7 +18339,7 @@
         <v>1</v>
       </c>
       <c r="P156" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="157">
@@ -18397,7 +18389,7 @@
         <v>1</v>
       </c>
       <c r="P157" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="158">
@@ -18735,7 +18727,7 @@
         <v>0</v>
       </c>
       <c r="P164" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="165">
@@ -18785,7 +18777,7 @@
         <v>0</v>
       </c>
       <c r="P165" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="166">
@@ -18931,7 +18923,7 @@
         <v>0</v>
       </c>
       <c r="P168" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="169">
@@ -18981,7 +18973,7 @@
         <v>0</v>
       </c>
       <c r="P169" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="170">
@@ -19580,7 +19572,7 @@
         <v>0</v>
       </c>
       <c r="G182" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H182" s="5" t="b">
         <v>0</v>
@@ -19607,7 +19599,7 @@
         <v>0</v>
       </c>
       <c r="P182" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="183">
@@ -19630,7 +19622,7 @@
         <v>0</v>
       </c>
       <c r="G183" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H183" s="5" t="b">
         <v>0</v>
@@ -19656,9 +19648,7 @@
       <c r="O183" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="P183" s="6" t="s">
-        <v>289</v>
-      </c>
+      <c r="P183" s="6"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="b">
@@ -19755,7 +19745,7 @@
         <v>1</v>
       </c>
       <c r="P185" s="6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="186">
@@ -19805,7 +19795,7 @@
         <v>1</v>
       </c>
       <c r="P186" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="187">
@@ -20031,8 +20021,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.13"/>
-    <col customWidth="1" min="2" max="2" width="7.25"/>
-    <col customWidth="1" min="3" max="3" width="9.88"/>
+    <col customWidth="1" min="2" max="2" width="8.0"/>
+    <col customWidth="1" min="3" max="3" width="11.0"/>
     <col customWidth="1" min="4" max="4" width="3.25"/>
     <col customWidth="1" min="5" max="5" width="7.0"/>
     <col customWidth="1" min="6" max="6" width="4.5"/>
@@ -20057,22 +20047,22 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>295</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>15</v>
@@ -21840,7 +21830,7 @@
         <v>0</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51">
@@ -21878,7 +21868,7 @@
         <v>0</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="52">
@@ -21952,7 +21942,7 @@
         <v>0</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54">
@@ -22242,7 +22232,7 @@
         <v>0</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="62">
@@ -22676,7 +22666,7 @@
         <v>0</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="74">
@@ -22786,7 +22776,7 @@
         <v>0</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="77">
@@ -23219,7 +23209,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="89">
@@ -23437,7 +23427,7 @@
         <v>0</v>
       </c>
       <c r="L94" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="95">
@@ -23943,7 +23933,7 @@
         <v>0</v>
       </c>
       <c r="L108" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="109">
@@ -24449,7 +24439,7 @@
         <v>0</v>
       </c>
       <c r="L122" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="123">
@@ -25063,7 +25053,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="140">
@@ -25821,7 +25811,7 @@
         <v>0</v>
       </c>
       <c r="L160" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="161">
@@ -26219,7 +26209,7 @@
         <v>0</v>
       </c>
       <c r="L171" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="172">
@@ -26509,7 +26499,7 @@
         <v>0</v>
       </c>
       <c r="L179" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="180">
@@ -27015,7 +27005,7 @@
         <v>0</v>
       </c>
       <c r="L193" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="194">
@@ -27449,7 +27439,7 @@
         <v>0</v>
       </c>
       <c r="L205" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="206">
@@ -27667,7 +27657,7 @@
         <v>0</v>
       </c>
       <c r="L211" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="212">
@@ -28173,7 +28163,7 @@
         <v>0</v>
       </c>
       <c r="L225" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="226">
@@ -28967,7 +28957,7 @@
         <v>0</v>
       </c>
       <c r="L247" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="248">
@@ -29041,7 +29031,7 @@
         <v>0</v>
       </c>
       <c r="L249" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="250">
@@ -29187,7 +29177,7 @@
         <v>0</v>
       </c>
       <c r="L253" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="254">
@@ -31348,7 +31338,7 @@
         <v>0</v>
       </c>
       <c r="L313" s="6" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="314">
@@ -31386,7 +31376,7 @@
         <v>0</v>
       </c>
       <c r="L314" s="6" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="315">
@@ -31852,8 +31842,8 @@
       <c r="J327" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K327" s="5" t="b">
-        <v>0</v>
+      <c r="K327" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L327" s="7"/>
     </row>
@@ -32108,7 +32098,7 @@
         <v>0</v>
       </c>
       <c r="L334" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="335">
@@ -32970,8 +32960,8 @@
       <c r="J358" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K358" s="5" t="b">
-        <v>0</v>
+      <c r="K358" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L358" s="7"/>
     </row>
@@ -33114,8 +33104,8 @@
       <c r="J362" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K362" s="5" t="b">
-        <v>0</v>
+      <c r="K362" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L362" s="7"/>
     </row>
@@ -33150,8 +33140,8 @@
       <c r="J363" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K363" s="5" t="b">
-        <v>0</v>
+      <c r="K363" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L363" s="7"/>
     </row>
@@ -33186,8 +33176,8 @@
       <c r="J364" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K364" s="5" t="b">
-        <v>0</v>
+      <c r="K364" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L364" s="7"/>
     </row>
@@ -33222,8 +33212,8 @@
       <c r="J365" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K365" s="5" t="b">
-        <v>0</v>
+      <c r="K365" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L365" s="7"/>
     </row>
@@ -33331,7 +33321,7 @@
         <v>0</v>
       </c>
       <c r="K368" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L368" s="7"/>
     </row>
@@ -33582,8 +33572,8 @@
       <c r="J375" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K375" s="5" t="b">
-        <v>0</v>
+      <c r="K375" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L375" s="7"/>
     </row>
@@ -33618,8 +33608,8 @@
       <c r="J376" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K376" s="5" t="b">
-        <v>0</v>
+      <c r="K376" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L376" s="7"/>
     </row>
@@ -33978,8 +33968,8 @@
       <c r="J386" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K386" s="5" t="b">
-        <v>0</v>
+      <c r="K386" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L386" s="7"/>
     </row>
@@ -34054,7 +34044,7 @@
         <v>0</v>
       </c>
       <c r="L388" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="389">
@@ -34196,8 +34186,8 @@
       <c r="J392" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K392" s="5" t="b">
-        <v>0</v>
+      <c r="K392" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L392" s="7"/>
     </row>
@@ -34484,8 +34474,8 @@
       <c r="J400" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K400" s="5" t="b">
-        <v>0</v>
+      <c r="K400" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L400" s="7"/>
     </row>
@@ -34700,8 +34690,8 @@
       <c r="J406" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K406" s="5" t="b">
-        <v>0</v>
+      <c r="K406" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L406" s="7"/>
     </row>
@@ -34736,8 +34726,8 @@
       <c r="J407" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K407" s="5" t="b">
-        <v>0</v>
+      <c r="K407" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L407" s="7"/>
     </row>
@@ -34772,8 +34762,8 @@
       <c r="J408" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K408" s="5" t="b">
-        <v>0</v>
+      <c r="K408" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L408" s="7"/>
     </row>
@@ -34884,7 +34874,7 @@
         <v>0</v>
       </c>
       <c r="L411" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="412">
@@ -35102,7 +35092,7 @@
         <v>0</v>
       </c>
       <c r="L417" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="418">
@@ -35172,8 +35162,8 @@
       <c r="J419" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K419" s="5" t="b">
-        <v>0</v>
+      <c r="K419" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L419" s="7"/>
     </row>
@@ -35208,8 +35198,8 @@
       <c r="J420" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K420" s="5" t="b">
-        <v>0</v>
+      <c r="K420" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L420" s="7"/>
     </row>
@@ -35320,7 +35310,7 @@
         <v>0</v>
       </c>
       <c r="L423" s="6" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="424">
@@ -35787,10 +35777,10 @@
         <v>0</v>
       </c>
       <c r="K436" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L436" s="6" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
     </row>
     <row r="437">
@@ -35824,8 +35814,8 @@
       <c r="J437" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K437" s="5" t="b">
-        <v>0</v>
+      <c r="K437" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L437" s="7"/>
     </row>
@@ -35968,8 +35958,8 @@
       <c r="J441" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K441" s="5" t="b">
-        <v>0</v>
+      <c r="K441" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L441" s="7"/>
     </row>
@@ -36004,8 +35994,8 @@
       <c r="J442" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K442" s="5" t="b">
-        <v>0</v>
+      <c r="K442" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L442" s="7"/>
     </row>
@@ -36080,7 +36070,7 @@
         <v>0</v>
       </c>
       <c r="L444" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="445">
@@ -36190,7 +36180,7 @@
         <v>0</v>
       </c>
       <c r="L447" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="448">
@@ -36444,7 +36434,7 @@
         <v>0</v>
       </c>
       <c r="L454" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="455">
@@ -36698,7 +36688,7 @@
         <v>0</v>
       </c>
       <c r="L461" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="462">
@@ -36952,7 +36942,7 @@
         <v>0</v>
       </c>
       <c r="L468" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="469">
@@ -37134,7 +37124,7 @@
         <v>0</v>
       </c>
       <c r="L473" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="474">
@@ -37244,7 +37234,7 @@
         <v>0</v>
       </c>
       <c r="L476" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="477">
@@ -37354,7 +37344,7 @@
         <v>0</v>
       </c>
       <c r="L479" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="480">
@@ -37388,8 +37378,8 @@
       <c r="J480" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K480" s="5" t="b">
-        <v>0</v>
+      <c r="K480" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L480" s="7"/>
     </row>
@@ -37496,8 +37486,8 @@
       <c r="J483" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K483" s="5" t="b">
-        <v>0</v>
+      <c r="K483" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L483" s="7"/>
     </row>
@@ -37532,8 +37522,8 @@
       <c r="J484" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K484" s="5" t="b">
-        <v>0</v>
+      <c r="K484" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L484" s="7"/>
     </row>
@@ -37640,8 +37630,8 @@
       <c r="J487" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K487" s="5" t="b">
-        <v>0</v>
+      <c r="K487" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L487" s="7"/>
     </row>
@@ -37784,8 +37774,8 @@
       <c r="J491" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K491" s="5" t="b">
-        <v>0</v>
+      <c r="K491" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L491" s="7"/>
     </row>
@@ -37820,8 +37810,8 @@
       <c r="J492" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K492" s="5" t="b">
-        <v>0</v>
+      <c r="K492" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L492" s="7"/>
     </row>
@@ -37856,8 +37846,8 @@
       <c r="J493" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K493" s="5" t="b">
-        <v>0</v>
+      <c r="K493" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L493" s="7"/>
     </row>
@@ -37928,8 +37918,8 @@
       <c r="J495" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K495" s="5" t="b">
-        <v>0</v>
+      <c r="K495" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L495" s="7"/>
     </row>
@@ -37964,8 +37954,8 @@
       <c r="J496" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K496" s="5" t="b">
-        <v>0</v>
+      <c r="K496" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L496" s="7"/>
     </row>
@@ -38000,8 +37990,8 @@
       <c r="J497" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K497" s="5" t="b">
-        <v>0</v>
+      <c r="K497" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L497" s="7"/>
     </row>
@@ -38036,8 +38026,8 @@
       <c r="J498" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K498" s="5" t="b">
-        <v>0</v>
+      <c r="K498" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L498" s="7"/>
     </row>
@@ -38072,8 +38062,8 @@
       <c r="J499" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K499" s="5" t="b">
-        <v>0</v>
+      <c r="K499" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L499" s="7"/>
     </row>
@@ -38108,8 +38098,8 @@
       <c r="J500" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K500" s="5" t="b">
-        <v>0</v>
+      <c r="K500" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L500" s="7"/>
     </row>
@@ -41276,8 +41266,8 @@
       <c r="J588" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K588" s="5" t="b">
-        <v>0</v>
+      <c r="K588" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L588" s="7"/>
     </row>
@@ -41348,8 +41338,8 @@
       <c r="J590" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K590" s="5" t="b">
-        <v>0</v>
+      <c r="K590" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L590" s="7"/>
     </row>
@@ -41420,8 +41410,8 @@
       <c r="J592" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K592" s="5" t="b">
-        <v>0</v>
+      <c r="K592" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L592" s="7"/>
     </row>
@@ -41492,8 +41482,8 @@
       <c r="J594" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K594" s="5" t="b">
-        <v>0</v>
+      <c r="K594" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L594" s="7"/>
     </row>
@@ -41529,10 +41519,10 @@
         <v>0</v>
       </c>
       <c r="K595" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L595" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="596">
@@ -41746,8 +41736,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="5.13"/>
-    <col customWidth="1" min="2" max="2" width="7.25"/>
-    <col customWidth="1" min="3" max="3" width="9.88"/>
+    <col customWidth="1" min="2" max="2" width="7.88"/>
+    <col customWidth="1" min="3" max="3" width="10.75"/>
     <col customWidth="1" min="4" max="4" width="3.25"/>
     <col customWidth="1" min="5" max="5" width="7.0"/>
     <col customWidth="1" min="6" max="6" width="4.5"/>
@@ -41772,22 +41762,22 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>295</v>
       </c>
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>15</v>
@@ -42260,7 +42250,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="15">
@@ -42298,7 +42288,7 @@
         <v>0</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16">
@@ -42336,7 +42326,7 @@
         <v>0</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="17">
@@ -43093,7 +43083,7 @@
         <v>0</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="38">
@@ -43563,7 +43553,7 @@
         <v>0</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="51">
@@ -43961,7 +43951,7 @@
         <v>0</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="62">
@@ -44035,7 +44025,7 @@
         <v>0</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="64">
@@ -44397,7 +44387,7 @@
         <v>0</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="74">
@@ -44507,7 +44497,7 @@
         <v>0</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="77">
@@ -44941,7 +44931,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="89">
@@ -45159,7 +45149,7 @@
         <v>0</v>
       </c>
       <c r="L94" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="95">
@@ -45233,7 +45223,7 @@
         <v>0</v>
       </c>
       <c r="L96" s="6" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
     </row>
     <row r="97">
@@ -45451,7 +45441,7 @@
         <v>0</v>
       </c>
       <c r="L102" s="6" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="103">
@@ -45669,7 +45659,7 @@
         <v>0</v>
       </c>
       <c r="L108" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="109">
@@ -45743,7 +45733,7 @@
         <v>0</v>
       </c>
       <c r="L110" s="6" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="111">
@@ -46177,7 +46167,7 @@
         <v>0</v>
       </c>
       <c r="L122" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="123">
@@ -46251,7 +46241,7 @@
         <v>0</v>
       </c>
       <c r="L124" s="6" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="125">
@@ -46541,7 +46531,7 @@
         <v>0</v>
       </c>
       <c r="L132" s="6" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="133">
@@ -46651,7 +46641,7 @@
         <v>0</v>
       </c>
       <c r="L135" s="6" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="136">
@@ -46797,7 +46787,7 @@
         <v>0</v>
       </c>
       <c r="L139" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="140">
@@ -47087,7 +47077,7 @@
         <v>0</v>
       </c>
       <c r="L147" s="6" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
     </row>
     <row r="148">
@@ -47197,7 +47187,7 @@
         <v>0</v>
       </c>
       <c r="L150" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="151">
@@ -47271,7 +47261,7 @@
         <v>0</v>
       </c>
       <c r="L152" s="6" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="153">
@@ -47417,7 +47407,7 @@
         <v>0</v>
       </c>
       <c r="L156" s="6" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="157">
@@ -47563,7 +47553,7 @@
         <v>0</v>
       </c>
       <c r="L160" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="161">
@@ -47961,7 +47951,7 @@
         <v>0</v>
       </c>
       <c r="L171" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="172">
@@ -48251,7 +48241,7 @@
         <v>0</v>
       </c>
       <c r="L179" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="180">
@@ -48757,7 +48747,7 @@
         <v>0</v>
       </c>
       <c r="L193" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="194">
@@ -48831,7 +48821,7 @@
         <v>0</v>
       </c>
       <c r="L195" s="6" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="196">
@@ -49193,7 +49183,7 @@
         <v>0</v>
       </c>
       <c r="L205" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="206">
@@ -49267,7 +49257,7 @@
         <v>0</v>
       </c>
       <c r="L207" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="208">
@@ -49413,7 +49403,7 @@
         <v>0</v>
       </c>
       <c r="L211" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="212">
@@ -49775,7 +49765,7 @@
         <v>0</v>
       </c>
       <c r="L221" s="6" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
     </row>
     <row r="222">
@@ -49921,7 +49911,7 @@
         <v>0</v>
       </c>
       <c r="L225" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="226">
@@ -49995,7 +49985,7 @@
         <v>0</v>
       </c>
       <c r="L227" s="6" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
     </row>
     <row r="228">
@@ -50213,7 +50203,7 @@
         <v>0</v>
       </c>
       <c r="L233" s="6" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="234">
@@ -50719,7 +50709,7 @@
         <v>0</v>
       </c>
       <c r="L247" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="248">
@@ -50793,7 +50783,7 @@
         <v>0</v>
       </c>
       <c r="L249" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="250">
@@ -50867,7 +50857,7 @@
         <v>0</v>
       </c>
       <c r="L251" s="6" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="252">
@@ -50941,7 +50931,7 @@
         <v>0</v>
       </c>
       <c r="L253" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="254">
@@ -51159,7 +51149,7 @@
         <v>0</v>
       </c>
       <c r="L259" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="260">
@@ -51197,7 +51187,7 @@
         <v>0</v>
       </c>
       <c r="L260" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="261">
@@ -51235,7 +51225,7 @@
         <v>0</v>
       </c>
       <c r="L261" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="262">
@@ -52029,7 +52019,7 @@
         <v>0</v>
       </c>
       <c r="L283" s="6" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="284">
@@ -52103,7 +52093,7 @@
         <v>0</v>
       </c>
       <c r="L285" s="6" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="286">
@@ -52717,7 +52707,7 @@
         <v>0</v>
       </c>
       <c r="L302" s="6" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="303">
@@ -52863,7 +52853,7 @@
         <v>0</v>
       </c>
       <c r="L306" s="6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="307">
@@ -53117,7 +53107,7 @@
         <v>0</v>
       </c>
       <c r="L313" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="314">
@@ -53155,7 +53145,7 @@
         <v>0</v>
       </c>
       <c r="L314" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="315">
@@ -53877,7 +53867,7 @@
         <v>0</v>
       </c>
       <c r="L334" s="6" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="335">
@@ -55067,7 +55057,7 @@
         <v>0</v>
       </c>
       <c r="L367" s="6" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="368">
@@ -55825,7 +55815,7 @@
         <v>0</v>
       </c>
       <c r="L388" s="6" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="389">
@@ -56043,7 +56033,7 @@
         <v>1</v>
       </c>
       <c r="L394" s="6" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="395">
@@ -56657,7 +56647,7 @@
         <v>0</v>
       </c>
       <c r="L411" s="6" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="412">
@@ -56875,7 +56865,7 @@
         <v>0</v>
       </c>
       <c r="L417" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="418">
@@ -57093,7 +57083,7 @@
         <v>0</v>
       </c>
       <c r="L423" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="424">
@@ -57851,7 +57841,7 @@
         <v>0</v>
       </c>
       <c r="L444" s="6" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="445">
@@ -57961,7 +57951,7 @@
         <v>0</v>
       </c>
       <c r="L447" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="448">
@@ -58215,7 +58205,7 @@
         <v>0</v>
       </c>
       <c r="L454" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="455">
@@ -58469,7 +58459,7 @@
         <v>0</v>
       </c>
       <c r="L461" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="462">
@@ -58723,7 +58713,7 @@
         <v>0</v>
       </c>
       <c r="L468" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="469">
@@ -58905,7 +58895,7 @@
         <v>0</v>
       </c>
       <c r="L473" s="6" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="474">
@@ -59015,7 +59005,7 @@
         <v>0</v>
       </c>
       <c r="L476" s="6" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="477">
@@ -59125,7 +59115,7 @@
         <v>0</v>
       </c>
       <c r="L479" s="6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="480">
@@ -59667,7 +59657,7 @@
         <v>0</v>
       </c>
       <c r="L494" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="495">
@@ -60101,7 +60091,7 @@
         <v>0</v>
       </c>
       <c r="L506" s="6" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="507">
@@ -63307,7 +63297,7 @@
         <v>1</v>
       </c>
       <c r="L595" s="6" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="596">
@@ -63528,16 +63518,16 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="I1" s="10" t="s">
         <v>340</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="I1" s="10" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1">
@@ -63563,37 +63553,37 @@
         <v>0</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="F3" s="14" t="s">
         <v>0</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="I3" s="10" t="s">
         <v>0</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K3" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="L3" s="14" t="s">
         <v>0</v>
       </c>
       <c r="M3" s="13" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="N3" s="13" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4">
@@ -63706,7 +63696,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="22">

</xml_diff>

<commit_message>
Finalized manually labeled data set
</commit_message>
<xml_diff>
--- a/data/labeling/rq4tlr-manual-variables.xlsx
+++ b/data/labeling/rq4tlr-manual-variables.xlsx
@@ -2240,7 +2240,7 @@
       <c r="H16" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="I16" s="5" t="b">
+      <c r="I16" s="4" t="b">
         <v>0</v>
       </c>
       <c r="J16" s="4" t="b">
@@ -22300,7 +22300,7 @@
         <v>0</v>
       </c>
       <c r="J63" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" s="4" t="b">
         <v>0</v>
@@ -23494,8 +23494,8 @@
       <c r="I96" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J96" s="5" t="b">
-        <v>0</v>
+      <c r="J96" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K96" s="5" t="b">
         <v>0</v>
@@ -23710,8 +23710,8 @@
       <c r="I102" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J102" s="5" t="b">
-        <v>0</v>
+      <c r="J102" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K102" s="5" t="b">
         <v>0</v>
@@ -24000,8 +24000,8 @@
       <c r="I110" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J110" s="5" t="b">
-        <v>0</v>
+      <c r="J110" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K110" s="5" t="b">
         <v>0</v>
@@ -24506,8 +24506,8 @@
       <c r="I124" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J124" s="5" t="b">
-        <v>0</v>
+      <c r="J124" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K124" s="5" t="b">
         <v>0</v>
@@ -24794,8 +24794,8 @@
       <c r="I132" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J132" s="5" t="b">
-        <v>0</v>
+      <c r="J132" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K132" s="5" t="b">
         <v>0</v>
@@ -24902,8 +24902,8 @@
       <c r="I135" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J135" s="5" t="b">
-        <v>0</v>
+      <c r="J135" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K135" s="5" t="b">
         <v>0</v>
@@ -25516,8 +25516,8 @@
       <c r="I152" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J152" s="5" t="b">
-        <v>0</v>
+      <c r="J152" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K152" s="5" t="b">
         <v>0</v>
@@ -27072,8 +27072,8 @@
       <c r="I195" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J195" s="5" t="b">
-        <v>0</v>
+      <c r="J195" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K195" s="5" t="b">
         <v>0</v>
@@ -27506,8 +27506,8 @@
       <c r="I207" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J207" s="5" t="b">
-        <v>0</v>
+      <c r="J207" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K207" s="5" t="b">
         <v>0</v>
@@ -28012,8 +28012,8 @@
       <c r="I221" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J221" s="5" t="b">
-        <v>0</v>
+      <c r="J221" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K221" s="5" t="b">
         <v>0</v>
@@ -28230,8 +28230,8 @@
       <c r="I227" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J227" s="5" t="b">
-        <v>0</v>
+      <c r="J227" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K227" s="5" t="b">
         <v>0</v>
@@ -28446,8 +28446,8 @@
       <c r="I233" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J233" s="5" t="b">
-        <v>0</v>
+      <c r="J233" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K233" s="5" t="b">
         <v>0</v>
@@ -29098,8 +29098,8 @@
       <c r="I251" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J251" s="5" t="b">
-        <v>0</v>
+      <c r="J251" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K251" s="5" t="b">
         <v>0</v>
@@ -29388,8 +29388,8 @@
       <c r="I259" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J259" s="5" t="b">
-        <v>0</v>
+      <c r="J259" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K259" s="5" t="b">
         <v>0</v>
@@ -29424,8 +29424,8 @@
       <c r="I260" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J260" s="5" t="b">
-        <v>0</v>
+      <c r="J260" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K260" s="5" t="b">
         <v>0</v>
@@ -29460,8 +29460,8 @@
       <c r="I261" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J261" s="5" t="b">
-        <v>0</v>
+      <c r="J261" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K261" s="5" t="b">
         <v>0</v>
@@ -30827,8 +30827,8 @@
       <c r="I299" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J299" s="5" t="b">
-        <v>0</v>
+      <c r="J299" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K299" s="5" t="b">
         <v>0</v>
@@ -31151,8 +31151,8 @@
       <c r="I308" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J308" s="5" t="b">
-        <v>0</v>
+      <c r="J308" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K308" s="5" t="b">
         <v>0</v>
@@ -31187,8 +31187,8 @@
       <c r="I309" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J309" s="5" t="b">
-        <v>0</v>
+      <c r="J309" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K309" s="5" t="b">
         <v>0</v>
@@ -32165,8 +32165,8 @@
       <c r="I336" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J336" s="5" t="b">
-        <v>0</v>
+      <c r="J336" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K336" s="5" t="b">
         <v>0</v>
@@ -33932,8 +33932,8 @@
       <c r="J385" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K385" s="5" t="b">
-        <v>0</v>
+      <c r="K385" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L385" s="7"/>
     </row>
@@ -34222,8 +34222,8 @@
       <c r="J393" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K393" s="5" t="b">
-        <v>0</v>
+      <c r="K393" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L393" s="7"/>
     </row>
@@ -34258,8 +34258,8 @@
       <c r="J394" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K394" s="5" t="b">
-        <v>0</v>
+      <c r="K394" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L394" s="6"/>
     </row>
@@ -34795,8 +34795,8 @@
       <c r="I409" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J409" s="5" t="b">
-        <v>0</v>
+      <c r="J409" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K409" s="5" t="b">
         <v>0</v>
@@ -35163,7 +35163,7 @@
         <v>0</v>
       </c>
       <c r="K419" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L419" s="7"/>
     </row>
@@ -37594,7 +37594,7 @@
       <c r="J486" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K486" s="5" t="b">
+      <c r="K486" s="4" t="b">
         <v>0</v>
       </c>
       <c r="L486" s="7"/>
@@ -38959,7 +38959,7 @@
       <c r="I524" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J524" s="5" t="b">
+      <c r="J524" s="4" t="b">
         <v>0</v>
       </c>
       <c r="K524" s="5" t="b">
@@ -38995,8 +38995,8 @@
       <c r="I525" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J525" s="5" t="b">
-        <v>0</v>
+      <c r="J525" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K525" s="5" t="b">
         <v>0</v>
@@ -39463,8 +39463,8 @@
       <c r="I538" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J538" s="5" t="b">
-        <v>0</v>
+      <c r="J538" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K538" s="5" t="b">
         <v>0</v>
@@ -39679,8 +39679,8 @@
       <c r="I544" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J544" s="5" t="b">
-        <v>0</v>
+      <c r="J544" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K544" s="5" t="b">
         <v>0</v>
@@ -40939,8 +40939,8 @@
       <c r="I579" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="J579" s="5" t="b">
-        <v>0</v>
+      <c r="J579" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="K579" s="5" t="b">
         <v>0</v>
@@ -59366,7 +59366,7 @@
         <v>0</v>
       </c>
       <c r="K486" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L486" s="7"/>
     </row>
@@ -59617,8 +59617,8 @@
       <c r="J493" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K493" s="5" t="b">
-        <v>0</v>
+      <c r="K493" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L493" s="7"/>
     </row>
@@ -59727,8 +59727,8 @@
       <c r="J496" s="5" t="b">
         <v>0</v>
       </c>
-      <c r="K496" s="5" t="b">
-        <v>0</v>
+      <c r="K496" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="L496" s="7"/>
     </row>

</xml_diff>